<commit_message>
Added openweather feeds, added monitor code for all feed traffic
</commit_message>
<xml_diff>
--- a/bu_WEATHER_FEED_CATALOG.xlsx
+++ b/bu_WEATHER_FEED_CATALOG.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/587ce551b77ccc82/Documents/PlatformIO/Projects/ESP32-Weather-Aggragator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{989E3563-8B0F-4FEE-90E3-6FC740B2CBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{448D9BAB-3B37-4AF8-ADC1-A39D7ABC6087}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{989E3563-8B0F-4FEE-90E3-6FC740B2CBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{910A851D-54D7-4C98-9559-47EFB2705F88}"/>
   <bookViews>
     <workbookView xWindow="43080" yWindow="-2910" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{962BD6D7-0243-4F9A-A79E-196D6F841A54}"/>
   </bookViews>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -3294,7 +3294,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -3303,7 +3303,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -8358,7 +8357,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{974D433A-5FD9-4F57-83FD-8ABC67A317BB}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{974D433A-5FD9-4F57-83FD-8ABC67A317BB}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" showAll="0">
@@ -8770,7 +8769,7 @@
       <c r="A4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4">
         <v>311</v>
       </c>
     </row>
@@ -8778,7 +8777,7 @@
       <c r="A5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5">
         <v>4</v>
       </c>
     </row>
@@ -8786,7 +8785,7 @@
       <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6">
         <v>5</v>
       </c>
     </row>
@@ -8794,7 +8793,7 @@
       <c r="A7" s="5" t="s">
         <v>466</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7">
         <v>16</v>
       </c>
     </row>
@@ -8802,7 +8801,7 @@
       <c r="A8" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8">
         <v>29</v>
       </c>
     </row>
@@ -8810,7 +8809,7 @@
       <c r="A9" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9">
         <v>5</v>
       </c>
     </row>
@@ -8818,7 +8817,7 @@
       <c r="A10" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10">
         <v>24</v>
       </c>
     </row>
@@ -8826,7 +8825,7 @@
       <c r="A11" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11">
         <v>17</v>
       </c>
     </row>
@@ -8834,7 +8833,7 @@
       <c r="A12" s="5" t="s">
         <v>919</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12">
         <v>411</v>
       </c>
     </row>
@@ -20136,7 +20135,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="355" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="355" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A355" s="2" t="s">
         <v>152</v>
       </c>
@@ -20166,7 +20165,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="356" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="356" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A356" s="2" t="s">
         <v>152</v>
       </c>
@@ -20196,7 +20195,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="357" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="357" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A357" s="2" t="s">
         <v>152</v>
       </c>
@@ -20226,7 +20225,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="358" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="358" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A358" s="2" t="s">
         <v>152</v>
       </c>
@@ -20256,7 +20255,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="359" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="359" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A359" s="2" t="s">
         <v>152</v>
       </c>
@@ -20286,7 +20285,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="360" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="360" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A360" s="2" t="s">
         <v>152</v>
       </c>
@@ -20316,7 +20315,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="361" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="361" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A361" s="2" t="s">
         <v>152</v>
       </c>
@@ -20346,7 +20345,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="362" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="362" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A362" s="2" t="s">
         <v>152</v>
       </c>
@@ -20376,7 +20375,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="363" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="363" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A363" s="2" t="s">
         <v>152</v>
       </c>
@@ -20406,7 +20405,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="364" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="364" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A364" s="2" t="s">
         <v>152</v>
       </c>
@@ -20436,7 +20435,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="365" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="365" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A365" s="2" t="s">
         <v>152</v>
       </c>
@@ -20466,7 +20465,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="366" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="366" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A366" s="2" t="s">
         <v>152</v>
       </c>
@@ -20496,7 +20495,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="367" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="367" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A367" s="2" t="s">
         <v>152</v>
       </c>
@@ -20526,7 +20525,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="368" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="368" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A368" s="2" t="s">
         <v>152</v>
       </c>
@@ -20556,7 +20555,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="369" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="369" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A369" s="2" t="s">
         <v>152</v>
       </c>
@@ -20586,7 +20585,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="370" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="370" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A370" s="2" t="s">
         <v>152</v>
       </c>
@@ -20616,7 +20615,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="371" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="371" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A371" s="2" t="s">
         <v>152</v>
       </c>
@@ -20646,7 +20645,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="372" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="372" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A372" s="2" t="s">
         <v>152</v>
       </c>
@@ -20676,7 +20675,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="373" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="373" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A373" s="2" t="s">
         <v>152</v>
       </c>
@@ -20706,7 +20705,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="374" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="374" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A374" s="2" t="s">
         <v>152</v>
       </c>
@@ -20736,7 +20735,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="375" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="375" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A375" s="2" t="s">
         <v>152</v>
       </c>
@@ -20766,7 +20765,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="376" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="376" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A376" s="2" t="s">
         <v>152</v>
       </c>
@@ -20796,7 +20795,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="377" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="377" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A377" s="2" t="s">
         <v>152</v>
       </c>
@@ -21300,7 +21299,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="394" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="394" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A394" s="2" t="s">
         <v>152</v>
       </c>
@@ -21328,7 +21327,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="395" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="395" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A395" s="2" t="s">
         <v>207</v>
       </c>
@@ -21356,7 +21355,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="396" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="396" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A396" s="2" t="s">
         <v>207</v>
       </c>
@@ -21386,7 +21385,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="397" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="397" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A397" s="2" t="s">
         <v>207</v>
       </c>
@@ -21416,7 +21415,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="398" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="398" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A398" s="2" t="s">
         <v>207</v>
       </c>
@@ -21446,7 +21445,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="399" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="399" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A399" s="2" t="s">
         <v>207</v>
       </c>
@@ -21476,7 +21475,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="400" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="400" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A400" s="2" t="s">
         <v>207</v>
       </c>
@@ -21506,7 +21505,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="401" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="401" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A401" s="2" t="s">
         <v>207</v>
       </c>
@@ -21536,7 +21535,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="402" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="402" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A402" s="2" t="s">
         <v>207</v>
       </c>
@@ -21566,7 +21565,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="403" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="403" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A403" s="2" t="s">
         <v>207</v>
       </c>
@@ -21596,7 +21595,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="404" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="404" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A404" s="2" t="s">
         <v>207</v>
       </c>
@@ -21626,7 +21625,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="405" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="405" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A405" s="2" t="s">
         <v>207</v>
       </c>
@@ -21656,7 +21655,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="406" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="406" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A406" s="2" t="s">
         <v>207</v>
       </c>
@@ -21686,7 +21685,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="407" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="407" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A407" s="2" t="s">
         <v>207</v>
       </c>
@@ -21716,7 +21715,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="408" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="408" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A408" s="2" t="s">
         <v>207</v>
       </c>
@@ -21746,7 +21745,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="409" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="409" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A409" s="2" t="s">
         <v>207</v>
       </c>
@@ -21776,7 +21775,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="410" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="410" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A410" s="2" t="s">
         <v>207</v>
       </c>
@@ -21806,7 +21805,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="411" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="411" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A411" s="2" t="s">
         <v>207</v>
       </c>
@@ -21872,7 +21871,7 @@
   <autoFilter ref="A1:J412" xr:uid="{9D61CBEE-D806-4C92-B6D4-2299793F4DB5}">
     <filterColumn colId="0">
       <filters>
-        <filter val="WAPI"/>
+        <filter val="Open_Weather"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>